<commit_message>
2.1.9: Improve to generate of enumeration class.
</commit_message>
<xml_diff>
--- a/meta/program/BlancoValueObjectClassStructure.xlsx
+++ b/meta/program/BlancoValueObjectClassStructure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10911"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tueda/data/webstorm/blanco/blancoValueObject/meta/program/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58A6DAB9-9A76-0A48-A700-75408E09E56C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BE297CE-C817-C441-9A6A-874F13EE9478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8920" yWindow="460" windowWidth="28300" windowHeight="17440" tabRatio="640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8920" yWindow="500" windowWidth="28300" windowHeight="17440" tabRatio="640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="valueObject" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="86">
   <si>
     <t>1.このバリューオブジェクト定義書は、blancoValueObjectが入力ファイルとして利用します。</t>
   </si>
@@ -405,6 +405,49 @@
   </si>
   <si>
     <t>デフォルト</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>enumeration</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>java.lang.Boolean</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>列挙型かどうか。通常は false。</t>
+    <rPh sb="0" eb="3">
+      <t xml:space="preserve">レッキョガタ </t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>constructorArgList</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>java.util.List&lt;blanco.cg.valueobject.BlancoCgField&gt;</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>new java.util.ArrayList&lt;blanco.cg.valueobject.BlancoCgField&gt;()</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>クラス定義に含めるコンストラクタの引数マップです。&lt;引数名, 型&gt; となります。</t>
+    <rPh sb="6" eb="7">
+      <t xml:space="preserve">フクメル </t>
+    </rPh>
+    <rPh sb="17" eb="19">
+      <t xml:space="preserve">ヒキスウ </t>
+    </rPh>
+    <rPh sb="26" eb="27">
+      <t xml:space="preserve">ヒキスウメイ </t>
+    </rPh>
+    <rPh sb="31" eb="32">
+      <t xml:space="preserve">カタ </t>
+    </rPh>
     <phoneticPr fontId="3"/>
   </si>
 </sst>
@@ -970,13 +1013,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1389,7 +1432,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
@@ -1585,20 +1628,20 @@
       <c r="A19" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="B19" s="56" t="s">
+      <c r="B19" s="57" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="57"/>
-      <c r="D19" s="57"/>
+      <c r="C19" s="58"/>
+      <c r="D19" s="58"/>
       <c r="E19" s="53"/>
       <c r="F19"/>
       <c r="G19"/>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="55"/>
-      <c r="B20" s="56"/>
-      <c r="C20" s="57"/>
-      <c r="D20" s="57"/>
+      <c r="B20" s="57"/>
+      <c r="C20" s="58"/>
+      <c r="D20" s="58"/>
       <c r="E20" s="53"/>
       <c r="F20"/>
       <c r="G20"/>
@@ -1650,7 +1693,7 @@
       <c r="C25" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="D25" s="58" t="s">
+      <c r="D25" s="56" t="s">
         <v>78</v>
       </c>
       <c r="E25" s="54" t="s">
@@ -1705,7 +1748,7 @@
     </row>
     <row r="29" spans="1:7" ht="15">
       <c r="A29" s="38">
-        <f t="shared" ref="A29:A43" si="0">A28+1</f>
+        <f t="shared" ref="A29:A45" si="0">A28+1</f>
         <v>3</v>
       </c>
       <c r="B29" s="39" t="s">
@@ -1993,20 +2036,60 @@
       <c r="F43" s="51"/>
       <c r="G43"/>
     </row>
-    <row r="44" spans="1:7">
-      <c r="A44" s="21"/>
-      <c r="B44" s="22"/>
-      <c r="C44" s="44"/>
-      <c r="D44" s="44"/>
-      <c r="E44" s="48"/>
-      <c r="F44" s="49"/>
+    <row r="44" spans="1:7" s="47" customFormat="1" ht="15" customHeight="1">
+      <c r="A44" s="38">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="B44" s="39" t="s">
+        <v>79</v>
+      </c>
+      <c r="C44" s="40" t="s">
+        <v>80</v>
+      </c>
+      <c r="D44" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="E44" s="50" t="s">
+        <v>81</v>
+      </c>
+      <c r="F44" s="51"/>
       <c r="G44"/>
     </row>
-    <row r="45" spans="1:7">
+    <row r="45" spans="1:7" s="47" customFormat="1" ht="15" customHeight="1">
+      <c r="A45" s="38">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="B45" s="45" t="s">
+        <v>82</v>
+      </c>
+      <c r="C45" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="D45" s="46" t="s">
+        <v>84</v>
+      </c>
+      <c r="E45" s="50" t="s">
+        <v>85</v>
+      </c>
+      <c r="F45" s="51"/>
       <c r="G45"/>
     </row>
+    <row r="46" spans="1:7">
+      <c r="A46" s="21"/>
+      <c r="B46" s="22"/>
+      <c r="C46" s="44"/>
+      <c r="D46" s="44"/>
+      <c r="E46" s="48"/>
+      <c r="F46" s="49"/>
+      <c r="G46"/>
+    </row>
+    <row r="47" spans="1:7">
+      <c r="G47"/>
+    </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="27">
     <mergeCell ref="A25:A26"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="C25:C26"/>
@@ -2022,7 +2105,7 @@
     <mergeCell ref="E40:F40"/>
     <mergeCell ref="E32:F32"/>
     <mergeCell ref="E31:F31"/>
-    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="E46:F46"/>
     <mergeCell ref="E33:F33"/>
     <mergeCell ref="E34:F34"/>
     <mergeCell ref="E35:F35"/>
@@ -2032,10 +2115,12 @@
     <mergeCell ref="E41:F41"/>
     <mergeCell ref="E42:F42"/>
     <mergeCell ref="E43:F43"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="E44:F44"/>
   </mergeCells>
   <phoneticPr fontId="3"/>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D58" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D60" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>型</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>